<commit_message>
added legend and example row
</commit_message>
<xml_diff>
--- a/colored_header.xlsx
+++ b/colored_header.xlsx
@@ -32,7 +32,7 @@
       <b val="1"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
@@ -41,8 +41,14 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="0000FF00"/>
-        <bgColor rgb="0000FF00"/>
+        <fgColor rgb="008ED973"/>
+        <bgColor rgb="008ED973"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFFF00"/>
+        <bgColor rgb="00FFFF00"/>
       </patternFill>
     </fill>
     <fill>
@@ -53,8 +59,8 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00CCFFCC"/>
-        <bgColor rgb="00CCFFCC"/>
+        <fgColor rgb="00D9EFCD"/>
+        <bgColor rgb="00D9EFCD"/>
       </patternFill>
     </fill>
   </fills>
@@ -76,18 +82,22 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -453,7 +463,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AN2"/>
+  <dimension ref="A1:AN7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -721,10 +731,8 @@
           <t>Oregon &amp; Washington Lakes</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
+      <c r="E2" t="n">
+        <v>0</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -828,6 +836,232 @@
       <c r="AM2" t="inlineStr"/>
       <c r="AN2" t="inlineStr"/>
     </row>
+    <row r="3">
+      <c r="A3" s="5" t="inlineStr">
+        <is>
+          <t>The above row is an example row. Delete it and this row before uploading. Also delete the colour legend below</t>
+        </is>
+      </c>
+      <c r="B3" s="5" t="inlineStr"/>
+      <c r="C3" s="5" t="inlineStr"/>
+      <c r="D3" s="5" t="inlineStr"/>
+      <c r="E3" s="5" t="inlineStr"/>
+      <c r="F3" s="5" t="inlineStr"/>
+      <c r="G3" s="5" t="inlineStr"/>
+      <c r="H3" s="5" t="inlineStr"/>
+      <c r="I3" s="5" t="inlineStr"/>
+      <c r="J3" s="5" t="inlineStr"/>
+      <c r="K3" s="5" t="inlineStr"/>
+      <c r="L3" s="5" t="inlineStr"/>
+      <c r="M3" s="5" t="inlineStr"/>
+      <c r="N3" s="5" t="inlineStr"/>
+      <c r="O3" s="5" t="inlineStr"/>
+      <c r="P3" s="5" t="inlineStr"/>
+      <c r="Q3" s="5" t="inlineStr"/>
+      <c r="R3" s="5" t="inlineStr"/>
+      <c r="S3" s="5" t="inlineStr"/>
+      <c r="T3" s="5" t="inlineStr"/>
+      <c r="U3" s="5" t="inlineStr"/>
+      <c r="V3" s="5" t="inlineStr"/>
+      <c r="W3" s="5" t="inlineStr"/>
+      <c r="X3" s="5" t="inlineStr"/>
+      <c r="Y3" s="5" t="inlineStr"/>
+      <c r="Z3" s="5" t="inlineStr"/>
+      <c r="AA3" s="5" t="inlineStr"/>
+      <c r="AB3" s="5" t="inlineStr"/>
+      <c r="AC3" s="5" t="inlineStr"/>
+      <c r="AD3" s="5" t="inlineStr"/>
+      <c r="AE3" s="5" t="inlineStr"/>
+      <c r="AF3" s="5" t="inlineStr"/>
+      <c r="AG3" s="5" t="inlineStr"/>
+      <c r="AH3" s="5" t="inlineStr"/>
+      <c r="AI3" s="5" t="inlineStr"/>
+      <c r="AJ3" s="5" t="inlineStr"/>
+      <c r="AK3" s="5" t="inlineStr"/>
+      <c r="AL3" s="5" t="inlineStr"/>
+      <c r="AM3" s="5" t="inlineStr"/>
+      <c r="AN3" s="5" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr"/>
+      <c r="B4" t="inlineStr"/>
+      <c r="C4" t="inlineStr"/>
+      <c r="D4" t="inlineStr"/>
+      <c r="E4" t="inlineStr"/>
+      <c r="F4" t="inlineStr"/>
+      <c r="G4" t="inlineStr"/>
+      <c r="H4" t="inlineStr"/>
+      <c r="I4" t="inlineStr"/>
+      <c r="J4" t="inlineStr"/>
+      <c r="K4" t="inlineStr"/>
+      <c r="L4" t="inlineStr"/>
+      <c r="M4" t="inlineStr"/>
+      <c r="N4" t="inlineStr"/>
+      <c r="O4" t="inlineStr"/>
+      <c r="P4" t="inlineStr"/>
+      <c r="Q4" t="inlineStr"/>
+      <c r="R4" t="inlineStr"/>
+      <c r="S4" t="inlineStr"/>
+      <c r="T4" t="inlineStr"/>
+      <c r="U4" t="inlineStr"/>
+      <c r="V4" t="inlineStr"/>
+      <c r="W4" t="inlineStr"/>
+      <c r="X4" t="inlineStr"/>
+      <c r="Y4" t="inlineStr"/>
+      <c r="Z4" t="inlineStr"/>
+      <c r="AA4" t="inlineStr"/>
+      <c r="AB4" t="inlineStr"/>
+      <c r="AC4" t="inlineStr"/>
+      <c r="AD4" t="inlineStr"/>
+      <c r="AE4" t="inlineStr"/>
+      <c r="AF4" t="inlineStr"/>
+      <c r="AG4" t="inlineStr"/>
+      <c r="AH4" t="inlineStr"/>
+      <c r="AI4" t="inlineStr"/>
+      <c r="AJ4" t="inlineStr"/>
+      <c r="AK4" t="inlineStr"/>
+      <c r="AL4" t="inlineStr"/>
+      <c r="AM4" t="inlineStr"/>
+      <c r="AN4" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="6" t="inlineStr"/>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> = Mandatory column</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr"/>
+      <c r="D5" t="inlineStr"/>
+      <c r="E5" t="inlineStr"/>
+      <c r="F5" t="inlineStr"/>
+      <c r="G5" t="inlineStr"/>
+      <c r="H5" t="inlineStr"/>
+      <c r="I5" t="inlineStr"/>
+      <c r="J5" t="inlineStr"/>
+      <c r="K5" t="inlineStr"/>
+      <c r="L5" t="inlineStr"/>
+      <c r="M5" t="inlineStr"/>
+      <c r="N5" t="inlineStr"/>
+      <c r="O5" t="inlineStr"/>
+      <c r="P5" t="inlineStr"/>
+      <c r="Q5" t="inlineStr"/>
+      <c r="R5" t="inlineStr"/>
+      <c r="S5" t="inlineStr"/>
+      <c r="T5" t="inlineStr"/>
+      <c r="U5" t="inlineStr"/>
+      <c r="V5" t="inlineStr"/>
+      <c r="W5" t="inlineStr"/>
+      <c r="X5" t="inlineStr"/>
+      <c r="Y5" t="inlineStr"/>
+      <c r="Z5" t="inlineStr"/>
+      <c r="AA5" t="inlineStr"/>
+      <c r="AB5" t="inlineStr"/>
+      <c r="AC5" t="inlineStr"/>
+      <c r="AD5" t="inlineStr"/>
+      <c r="AE5" t="inlineStr"/>
+      <c r="AF5" t="inlineStr"/>
+      <c r="AG5" t="inlineStr"/>
+      <c r="AH5" t="inlineStr"/>
+      <c r="AI5" t="inlineStr"/>
+      <c r="AJ5" t="inlineStr"/>
+      <c r="AK5" t="inlineStr"/>
+      <c r="AL5" t="inlineStr"/>
+      <c r="AM5" t="inlineStr"/>
+      <c r="AN5" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="7" t="inlineStr"/>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> = Non-mandatory column</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr"/>
+      <c r="D6" t="inlineStr"/>
+      <c r="E6" t="inlineStr"/>
+      <c r="F6" t="inlineStr"/>
+      <c r="G6" t="inlineStr"/>
+      <c r="H6" t="inlineStr"/>
+      <c r="I6" t="inlineStr"/>
+      <c r="J6" t="inlineStr"/>
+      <c r="K6" t="inlineStr"/>
+      <c r="L6" t="inlineStr"/>
+      <c r="M6" t="inlineStr"/>
+      <c r="N6" t="inlineStr"/>
+      <c r="O6" t="inlineStr"/>
+      <c r="P6" t="inlineStr"/>
+      <c r="Q6" t="inlineStr"/>
+      <c r="R6" t="inlineStr"/>
+      <c r="S6" t="inlineStr"/>
+      <c r="T6" t="inlineStr"/>
+      <c r="U6" t="inlineStr"/>
+      <c r="V6" t="inlineStr"/>
+      <c r="W6" t="inlineStr"/>
+      <c r="X6" t="inlineStr"/>
+      <c r="Y6" t="inlineStr"/>
+      <c r="Z6" t="inlineStr"/>
+      <c r="AA6" t="inlineStr"/>
+      <c r="AB6" t="inlineStr"/>
+      <c r="AC6" t="inlineStr"/>
+      <c r="AD6" t="inlineStr"/>
+      <c r="AE6" t="inlineStr"/>
+      <c r="AF6" t="inlineStr"/>
+      <c r="AG6" t="inlineStr"/>
+      <c r="AH6" t="inlineStr"/>
+      <c r="AI6" t="inlineStr"/>
+      <c r="AJ6" t="inlineStr"/>
+      <c r="AK6" t="inlineStr"/>
+      <c r="AL6" t="inlineStr"/>
+      <c r="AM6" t="inlineStr"/>
+      <c r="AN6" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="8" t="inlineStr"/>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> = Mandatory depending on environment, type or other features</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr"/>
+      <c r="D7" t="inlineStr"/>
+      <c r="E7" t="inlineStr"/>
+      <c r="F7" t="inlineStr"/>
+      <c r="G7" t="inlineStr"/>
+      <c r="H7" t="inlineStr"/>
+      <c r="I7" t="inlineStr"/>
+      <c r="J7" t="inlineStr"/>
+      <c r="K7" t="inlineStr"/>
+      <c r="L7" t="inlineStr"/>
+      <c r="M7" t="inlineStr"/>
+      <c r="N7" t="inlineStr"/>
+      <c r="O7" t="inlineStr"/>
+      <c r="P7" t="inlineStr"/>
+      <c r="Q7" t="inlineStr"/>
+      <c r="R7" t="inlineStr"/>
+      <c r="S7" t="inlineStr"/>
+      <c r="T7" t="inlineStr"/>
+      <c r="U7" t="inlineStr"/>
+      <c r="V7" t="inlineStr"/>
+      <c r="W7" t="inlineStr"/>
+      <c r="X7" t="inlineStr"/>
+      <c r="Y7" t="inlineStr"/>
+      <c r="Z7" t="inlineStr"/>
+      <c r="AA7" t="inlineStr"/>
+      <c r="AB7" t="inlineStr"/>
+      <c r="AC7" t="inlineStr"/>
+      <c r="AD7" t="inlineStr"/>
+      <c r="AE7" t="inlineStr"/>
+      <c r="AF7" t="inlineStr"/>
+      <c r="AG7" t="inlineStr"/>
+      <c r="AH7" t="inlineStr"/>
+      <c r="AI7" t="inlineStr"/>
+      <c r="AJ7" t="inlineStr"/>
+      <c r="AK7" t="inlineStr"/>
+      <c r="AL7" t="inlineStr"/>
+      <c r="AM7" t="inlineStr"/>
+      <c r="AN7" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>